<commit_message>
Consolidate Dagster pipeline, LabBank Streamlit app, and optimization work
Single checkpoint commit capturing everything built since "before dagster":
the Dagster orchestration layer, the LabBank Streamlit sandbox app, the
bs_optimization module (4 optimizers), current README, pyproject.toml, and
accumulated fixes across optimize_prep/cash_flow_calc/irrbb_calc/ir_derivatives.

Also includes this session's GitHub-publish prep work:
- labbank_data_job (Dagster): regenerate a custom balance sheet and refresh
  LabBank's npz tensors in one job.
- "Reload my data" button in the LabBank app to pick up regenerated data
  without restarting Streamlit.
- .gitignore: exclude Dagster tmp run dirs and the copyrighted reference PDF.
- MIT LICENSE.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/irrbb_calc/output/eve_results.xlsx
+++ b/irrbb_calc/output/eve_results.xlsx
@@ -458,13 +458,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>-5837029699.068525</v>
+        <v>-6875102919.94</v>
       </c>
       <c r="D2" t="n">
-        <v>-161844533.8616113</v>
+        <v>-95696510.04890218</v>
       </c>
       <c r="E2" t="n">
-        <v>-5998874232.930137</v>
+        <v>-6970799429.988902</v>
       </c>
     </row>
     <row r="3">
@@ -479,13 +479,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1278847057.85</v>
+        <v>1284728808.5</v>
       </c>
       <c r="D3" t="n">
-        <v>231584150.3581635</v>
+        <v>317328976.2060196</v>
       </c>
       <c r="E3" t="n">
-        <v>1510431208.208163</v>
+        <v>1602057784.706019</v>
       </c>
     </row>
     <row r="4">
@@ -503,10 +503,10 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>-14336961.1800304</v>
+        <v>-8477827.203162251</v>
       </c>
       <c r="E4" t="n">
-        <v>-14336961.1800304</v>
+        <v>-8477827.203162251</v>
       </c>
     </row>
     <row r="5">
@@ -521,13 +521,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>5233457764.944227</v>
+        <v>5736321506.339336</v>
       </c>
       <c r="D5" t="n">
-        <v>1693640251.583912</v>
+        <v>1815154595.930524</v>
       </c>
       <c r="E5" t="n">
-        <v>6927098016.528139</v>
+        <v>7551476102.26986</v>
       </c>
     </row>
   </sheetData>
@@ -573,13 +573,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>675275123.7257019</v>
+        <v>145947394.8993364</v>
       </c>
       <c r="C2" t="n">
-        <v>1749042906.900434</v>
+        <v>2028309234.884479</v>
       </c>
       <c r="D2" t="n">
-        <v>2424318030.626136</v>
+        <v>2174256629.783815</v>
       </c>
     </row>
   </sheetData>
@@ -655,13 +655,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>-2695465919.310573</v>
+        <v>-3256778657.306471</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>-2695465919.310573</v>
+        <v>-3256778657.306471</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -669,7 +669,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>-2695465919.310573</v>
+        <v>-3256778657.306471</v>
       </c>
     </row>
     <row r="3">
@@ -689,13 +689,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>-1459014759.962479</v>
+        <v>-1763198912.999988</v>
       </c>
       <c r="E3" t="n">
-        <v>-86735165.71982653</v>
+        <v>-21094459.78994248</v>
       </c>
       <c r="F3" t="n">
-        <v>-1545749925.682306</v>
+        <v>-1784293372.78993</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -703,7 +703,7 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>-1545749925.682306</v>
+        <v>-1784293372.78993</v>
       </c>
     </row>
     <row r="4">
@@ -723,13 +723,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>-1444967479.344626</v>
+        <v>-1641504292.978168</v>
       </c>
       <c r="E4" t="n">
-        <v>-101462878.7715522</v>
+        <v>-102234344.4614767</v>
       </c>
       <c r="F4" t="n">
-        <v>-1546430358.116178</v>
+        <v>-1743738637.439645</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -737,7 +737,7 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>-1546430358.116178</v>
+        <v>-1743738637.439645</v>
       </c>
     </row>
     <row r="5">
@@ -757,13 +757,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>884354622.0529087</v>
+        <v>956644164.5950364</v>
       </c>
       <c r="E5" t="n">
-        <v>181942076.7411945</v>
+        <v>222153197.0988902</v>
       </c>
       <c r="F5" t="n">
-        <v>1066296698.794103</v>
+        <v>1178797361.693927</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -771,7 +771,7 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>1066296698.794103</v>
+        <v>1178797361.693927</v>
       </c>
     </row>
     <row r="6">
@@ -791,13 +791,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>317529440.6810989</v>
+        <v>225848751.8600489</v>
       </c>
       <c r="E6" t="n">
-        <v>51020927.52694491</v>
+        <v>111976446.1441714</v>
       </c>
       <c r="F6" t="n">
-        <v>368550368.2080438</v>
+        <v>337825198.0042203</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -805,7 +805,7 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>368550368.2080438</v>
+        <v>337825198.0042203</v>
       </c>
     </row>
     <row r="7">
@@ -828,10 +828,10 @@
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>189032198.9218521</v>
+        <v>48394700.73572497</v>
       </c>
       <c r="F7" t="n">
-        <v>189032198.9218521</v>
+        <v>48394700.73572497</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -839,7 +839,7 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>189032198.9218521</v>
+        <v>48394700.73572497</v>
       </c>
     </row>
     <row r="8">
@@ -862,10 +862,10 @@
         <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>-284716169.7502007</v>
+        <v>-79021734.3724252</v>
       </c>
       <c r="F8" t="n">
-        <v>-284716169.7502007</v>
+        <v>-79021734.3724252</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -873,7 +873,7 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>-284716169.7502007</v>
+        <v>-79021734.3724252</v>
       </c>
     </row>
     <row r="9">
@@ -893,13 +893,13 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1764517613.794478</v>
+        <v>1285144839.243104</v>
       </c>
       <c r="E9" t="n">
-        <v>545265787.1551471</v>
+        <v>371829556.977418</v>
       </c>
       <c r="F9" t="n">
-        <v>2309783400.949625</v>
+        <v>1656974396.220522</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -907,7 +907,7 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>2309783400.949625</v>
+        <v>1656974396.220522</v>
       </c>
     </row>
     <row r="10">
@@ -927,13 +927,13 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>3098391674.511272</v>
+        <v>4049592445.46318</v>
       </c>
       <c r="E10" t="n">
-        <v>1329884892.779564</v>
+        <v>1681127984.795213</v>
       </c>
       <c r="F10" t="n">
-        <v>4428276567.290836</v>
+        <v>5730720430.258393</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -941,7 +941,7 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>4428276567.290836</v>
+        <v>5730720430.258393</v>
       </c>
     </row>
     <row r="11">
@@ -961,13 +961,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>-3004287080.358242</v>
+        <v>-3583423798.486528</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>-3004287080.358242</v>
+        <v>-3583423798.486528</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -975,7 +975,7 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>-3004287080.358242</v>
+        <v>-3583423798.486528</v>
       </c>
     </row>
     <row r="12">
@@ -995,13 +995,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>-1547967289.521232</v>
+        <v>-1785341587.331126</v>
       </c>
       <c r="E12" t="n">
-        <v>-89974597.74089299</v>
+        <v>-21446988.5773839</v>
       </c>
       <c r="F12" t="n">
-        <v>-1637941887.262125</v>
+        <v>-1806788575.90851</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -1009,7 +1009,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>-1637941887.262125</v>
+        <v>-1806788575.90851</v>
       </c>
     </row>
     <row r="13">
@@ -1029,13 +1029,13 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>-1542214172.839975</v>
+        <v>-1739236876.100953</v>
       </c>
       <c r="E13" t="n">
-        <v>-44136590.95281409</v>
+        <v>-44790854.62068366</v>
       </c>
       <c r="F13" t="n">
-        <v>-1586350763.792789</v>
+        <v>-1784027730.721637</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -1043,7 +1043,7 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>-1586350763.792789</v>
+        <v>-1784027730.721637</v>
       </c>
     </row>
     <row r="14">
@@ -1063,13 +1063,13 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1016494720.626164</v>
+        <v>1104221921.89758</v>
       </c>
       <c r="E14" t="n">
-        <v>200633258.7332544</v>
+        <v>244067509.8078884</v>
       </c>
       <c r="F14" t="n">
-        <v>1217127979.359418</v>
+        <v>1348289431.705469</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1077,7 +1077,7 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>1217127979.359418</v>
+        <v>1348289431.705469</v>
       </c>
     </row>
     <row r="15">
@@ -1097,13 +1097,13 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>345848757.3690892</v>
+        <v>293779851.1165479</v>
       </c>
       <c r="E15" t="n">
-        <v>29333222.07038736</v>
+        <v>52898352.51548136</v>
       </c>
       <c r="F15" t="n">
-        <v>375181979.4394766</v>
+        <v>346678203.6320292</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1111,7 +1111,7 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>375181979.4394766</v>
+        <v>346678203.6320292</v>
       </c>
     </row>
     <row r="16">
@@ -1134,10 +1134,10 @@
         <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>202242745.6677688</v>
+        <v>52406121.7652897</v>
       </c>
       <c r="F16" t="n">
-        <v>202242745.6677688</v>
+        <v>52406121.7652897</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1145,7 +1145,7 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>202242745.6677688</v>
+        <v>52406121.7652897</v>
       </c>
     </row>
     <row r="17">
@@ -1168,10 +1168,10 @@
         <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>-130116086.0134829</v>
+        <v>-37113337.26254971</v>
       </c>
       <c r="F17" t="n">
-        <v>-130116086.0134829</v>
+        <v>-37113337.26254971</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1179,7 +1179,7 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>-130116086.0134829</v>
+        <v>-37113337.26254971</v>
       </c>
     </row>
     <row r="18">
@@ -1199,13 +1199,13 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>2012072973.872798</v>
+        <v>1461071018.42212</v>
       </c>
       <c r="E18" t="n">
-        <v>601658611.9384332</v>
+        <v>409610981.5324987</v>
       </c>
       <c r="F18" t="n">
-        <v>2613731585.811231</v>
+        <v>1870681999.954619</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1213,7 +1213,7 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>2613731585.811231</v>
+        <v>1870681999.954619</v>
       </c>
     </row>
     <row r="19">
@@ -1233,13 +1233,13 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>3636496095.83037</v>
+        <v>4724371980.772829</v>
       </c>
       <c r="E19" t="n">
-        <v>884850195.0321769</v>
+        <v>1136138637.676569</v>
       </c>
       <c r="F19" t="n">
-        <v>4521346290.862547</v>
+        <v>5860510618.449398</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1247,7 +1247,7 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>4521346290.862547</v>
+        <v>5860510618.449398</v>
       </c>
     </row>
     <row r="20">
@@ -1267,13 +1267,13 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>-2774441796.51401</v>
+        <v>-3340433482.509024</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>-2774441796.51401</v>
+        <v>-3340433482.509024</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1281,7 +1281,7 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>-2774441796.51401</v>
+        <v>-3340433482.509024</v>
       </c>
     </row>
     <row r="21">
@@ -1301,13 +1301,13 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>-1496460323.905028</v>
+        <v>-1779809062.420523</v>
       </c>
       <c r="E21" t="n">
-        <v>-88382304.60151681</v>
+        <v>-21351087.73845858</v>
       </c>
       <c r="F21" t="n">
-        <v>-1584842628.506545</v>
+        <v>-1801160150.158982</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1315,7 +1315,7 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>-1584842628.506545</v>
+        <v>-1801160150.158982</v>
       </c>
     </row>
     <row r="22">
@@ -1335,13 +1335,13 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>-1477214337.526204</v>
+        <v>-1674355105.551094</v>
       </c>
       <c r="E22" t="n">
-        <v>-82593056.79185569</v>
+        <v>-83373459.93998522</v>
       </c>
       <c r="F22" t="n">
-        <v>-1559807394.31806</v>
+        <v>-1757728565.491079</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1349,7 +1349,7 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>-1559807394.31806</v>
+        <v>-1757728565.491079</v>
       </c>
     </row>
     <row r="23">
@@ -1369,13 +1369,13 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>919157170.8797625</v>
+        <v>995367131.5699601</v>
       </c>
       <c r="E23" t="n">
-        <v>187716428.0752255</v>
+        <v>228842881.5594109</v>
       </c>
       <c r="F23" t="n">
-        <v>1106873598.954988</v>
+        <v>1224210013.129371</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1383,7 +1383,7 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>1106873598.954988</v>
+        <v>1224210013.129371</v>
       </c>
     </row>
     <row r="24">
@@ -1403,13 +1403,13 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>326430163.2321123</v>
+        <v>240541711.6625783</v>
       </c>
       <c r="E24" t="n">
-        <v>46857798.96902738</v>
+        <v>103117791.2761761</v>
       </c>
       <c r="F24" t="n">
-        <v>373287962.2011397</v>
+        <v>343659502.9387544</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -1417,7 +1417,7 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>373287962.2011397</v>
+        <v>343659502.9387544</v>
       </c>
     </row>
     <row r="25">
@@ -1440,10 +1440,10 @@
         <v>0</v>
       </c>
       <c r="E25" t="n">
-        <v>193967840.6387744</v>
+        <v>49778513.82820629</v>
       </c>
       <c r="F25" t="n">
-        <v>193967840.6387744</v>
+        <v>49778513.82820629</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -1451,7 +1451,7 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>193967840.6387744</v>
+        <v>49778513.82820629</v>
       </c>
     </row>
     <row r="26">
@@ -1474,10 +1474,10 @@
         <v>0</v>
       </c>
       <c r="E26" t="n">
-        <v>-244585457.4665864</v>
+        <v>-70044998.98962246</v>
       </c>
       <c r="F26" t="n">
-        <v>-244585457.4665864</v>
+        <v>-70044998.98962246</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -1485,7 +1485,7 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>-244585457.4665864</v>
+        <v>-70044998.98962246</v>
       </c>
     </row>
     <row r="27">
@@ -1505,13 +1505,13 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>1829965788.967272</v>
+        <v>1332083568.712087</v>
       </c>
       <c r="E27" t="n">
-        <v>562080426.4404492</v>
+        <v>383177640.415179</v>
       </c>
       <c r="F27" t="n">
-        <v>2392046215.407722</v>
+        <v>1715261209.127266</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -1519,7 +1519,7 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>2392046215.407722</v>
+        <v>1715261209.127266</v>
       </c>
     </row>
     <row r="28">
@@ -1539,13 +1539,13 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>3230946282.104176</v>
+        <v>4218012179.786539</v>
       </c>
       <c r="E28" t="n">
-        <v>1245099552.936992</v>
+        <v>1576812847.361132</v>
       </c>
       <c r="F28" t="n">
-        <v>4476045835.041168</v>
+        <v>5794825027.147671</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1553,7 +1553,7 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>4476045835.041168</v>
+        <v>5794825027.147671</v>
       </c>
     </row>
     <row r="29">
@@ -1573,13 +1573,13 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>-2898069824.98115</v>
+        <v>-3470957552.689276</v>
       </c>
       <c r="E29" t="n">
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>-2898069824.98115</v>
+        <v>-3470957552.689276</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -1587,7 +1587,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>-2898069824.98115</v>
+        <v>-3470957552.689276</v>
       </c>
     </row>
     <row r="30">
@@ -1607,13 +1607,13 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>-1503579610.51945</v>
+        <v>-1766716057.859257</v>
       </c>
       <c r="E30" t="n">
-        <v>-88065414.00512807</v>
+        <v>-21158734.396371</v>
       </c>
       <c r="F30" t="n">
-        <v>-1591645024.524578</v>
+        <v>-1787874792.255628</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1621,7 +1621,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>-1591645024.524578</v>
+        <v>-1787874792.255628</v>
       </c>
     </row>
     <row r="31">
@@ -1641,13 +1641,13 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>-1502359923.258183</v>
+        <v>-1698723691.342683</v>
       </c>
       <c r="E31" t="n">
-        <v>-67319034.01998186</v>
+        <v>-68138447.22528417</v>
       </c>
       <c r="F31" t="n">
-        <v>-1569678957.278165</v>
+        <v>-1766862138.567967</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1655,7 +1655,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>-1569678957.278165</v>
+        <v>-1766862138.567967</v>
       </c>
     </row>
     <row r="32">
@@ -1675,13 +1675,13 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>970674640.790839</v>
+        <v>1053022052.113768</v>
       </c>
       <c r="E32" t="n">
-        <v>193349948.7689836</v>
+        <v>235590924.785206</v>
       </c>
       <c r="F32" t="n">
-        <v>1164024589.559823</v>
+        <v>1288612976.898974</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -1689,7 +1689,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>1164024589.559823</v>
+        <v>1288612976.898974</v>
       </c>
     </row>
     <row r="33">
@@ -1709,13 +1709,13 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>334735585.8661783</v>
+        <v>272612670.7094528</v>
       </c>
       <c r="E33" t="n">
-        <v>35116708.9503255</v>
+        <v>67466217.2764869</v>
       </c>
       <c r="F33" t="n">
-        <v>369852294.8165038</v>
+        <v>340078887.9859397</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -1723,7 +1723,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>369852294.8165038</v>
+        <v>340078887.9859397</v>
       </c>
     </row>
     <row r="34">
@@ -1746,10 +1746,10 @@
         <v>0</v>
       </c>
       <c r="E34" t="n">
-        <v>196275252.2720836</v>
+        <v>50710365.60704952</v>
       </c>
       <c r="F34" t="n">
-        <v>196275252.2720836</v>
+        <v>50710365.60704952</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -1757,7 +1757,7 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>196275252.2720836</v>
+        <v>50710365.60704952</v>
       </c>
     </row>
     <row r="35">
@@ -1780,10 +1780,10 @@
         <v>0</v>
       </c>
       <c r="E35" t="n">
-        <v>-181907699.0576614</v>
+        <v>-49260503.18581253</v>
       </c>
       <c r="F35" t="n">
-        <v>-181907699.0576614</v>
+        <v>-49260503.18581253</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -1791,7 +1791,7 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>-181907699.0576614</v>
+        <v>-49260503.18581253</v>
       </c>
     </row>
     <row r="36">
@@ -1811,13 +1811,13 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>1924918822.438825</v>
+        <v>1398775318.730009</v>
       </c>
       <c r="E36" t="n">
-        <v>580140458.7122216</v>
+        <v>395116885.5672703</v>
       </c>
       <c r="F36" t="n">
-        <v>2505059281.151046</v>
+        <v>1793892204.29728</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -1825,7 +1825,7 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>2505059281.151046</v>
+        <v>1793892204.29728</v>
       </c>
     </row>
     <row r="37">
@@ -1845,13 +1845,13 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>3452874622.446946</v>
+        <v>4492948496.507627</v>
       </c>
       <c r="E37" t="n">
-        <v>1011312201.184338</v>
+        <v>1290648058.261173</v>
       </c>
       <c r="F37" t="n">
-        <v>4464186823.631284</v>
+        <v>5783596554.768801</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -1859,7 +1859,7 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>4464186823.631284</v>
+        <v>5783596554.768801</v>
       </c>
     </row>
     <row r="38">
@@ -1879,13 +1879,13 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>-2828980981.514099</v>
+        <v>-3397896505.289096</v>
       </c>
       <c r="E38" t="n">
         <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>-2828980981.514099</v>
+        <v>-3397896505.289096</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -1893,7 +1893,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>-2828980981.514099</v>
+        <v>-3397896505.289096</v>
       </c>
     </row>
     <row r="39">
@@ -1913,13 +1913,13 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>-1485719149.512565</v>
+        <v>-1763112731.422296</v>
       </c>
       <c r="E39" t="n">
-        <v>-87448574.21145189</v>
+        <v>-21100499.66340495</v>
       </c>
       <c r="F39" t="n">
-        <v>-1573167723.724016</v>
+        <v>-1784213231.085701</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -1927,7 +1927,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>-1573167723.724016</v>
+        <v>-1784213231.085701</v>
       </c>
     </row>
     <row r="40">
@@ -1947,13 +1947,13 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>-1481693248.090842</v>
+        <v>-1678005603.809977</v>
       </c>
       <c r="E40" t="n">
-        <v>-79563595.75534216</v>
+        <v>-80368350.91645695</v>
       </c>
       <c r="F40" t="n">
-        <v>-1561256843.846184</v>
+        <v>-1758373954.726434</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -1961,7 +1961,7 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>-1561256843.846184</v>
+        <v>-1758373954.726434</v>
       </c>
     </row>
     <row r="41">
@@ -1981,13 +1981,13 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>941315241.1942489</v>
+        <v>1020206080.940479</v>
       </c>
       <c r="E41" t="n">
-        <v>189315182.4043921</v>
+        <v>230847513.6164317</v>
       </c>
       <c r="F41" t="n">
-        <v>1130630423.598641</v>
+        <v>1251053594.556911</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
@@ -1995,7 +1995,7 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>1130630423.598641</v>
+        <v>1251053594.556911</v>
       </c>
     </row>
     <row r="42">
@@ -2015,13 +2015,13 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>328643044.2391157</v>
+        <v>256991512.47607</v>
       </c>
       <c r="E42" t="n">
-        <v>40103653.90342262</v>
+        <v>81556417.10022967</v>
       </c>
       <c r="F42" t="n">
-        <v>368746698.1425383</v>
+        <v>338547929.5762996</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -2029,7 +2029,7 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>368746698.1425383</v>
+        <v>338547929.5762996</v>
       </c>
     </row>
     <row r="43">
@@ -2052,10 +2052,10 @@
         <v>0</v>
       </c>
       <c r="E43" t="n">
-        <v>193540206.4021482</v>
+        <v>49865323.80716262</v>
       </c>
       <c r="F43" t="n">
-        <v>193540206.4021482</v>
+        <v>49865323.80716262</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -2063,7 +2063,7 @@
         </is>
       </c>
       <c r="H43" t="n">
-        <v>193540206.4021482</v>
+        <v>49865323.80716262</v>
       </c>
     </row>
     <row r="44">
@@ -2086,10 +2086,10 @@
         <v>0</v>
       </c>
       <c r="E44" t="n">
-        <v>-216063735.8948217</v>
+        <v>-58772444.62583864</v>
       </c>
       <c r="F44" t="n">
-        <v>-216063735.8948217</v>
+        <v>-58772444.62583864</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -2097,7 +2097,7 @@
         </is>
       </c>
       <c r="H44" t="n">
-        <v>-216063735.8948217</v>
+        <v>-58772444.62583864</v>
       </c>
     </row>
     <row r="45">
@@ -2117,13 +2117,13 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>1869848788.996442</v>
+        <v>1359702828.361849</v>
       </c>
       <c r="E45" t="n">
-        <v>567869159.9707233</v>
+        <v>386906886.3134878</v>
       </c>
       <c r="F45" t="n">
-        <v>2437717948.967165</v>
+        <v>1746609714.675337</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -2131,7 +2131,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>2437717948.967165</v>
+        <v>1746609714.675337</v>
       </c>
     </row>
     <row r="46">
@@ -2151,13 +2151,13 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>3331606199.803592</v>
+        <v>4341254252.794787</v>
       </c>
       <c r="E46" t="n">
-        <v>1114628303.452248</v>
+        <v>1417025437.412105</v>
       </c>
       <c r="F46" t="n">
-        <v>4446234503.255839</v>
+        <v>5758279690.206892</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -2165,7 +2165,7 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>4446234503.255839</v>
+        <v>5758279690.206892</v>
       </c>
     </row>
     <row r="47">
@@ -2185,13 +2185,13 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>-2855268888.074034</v>
+        <v>-3425924546.32583</v>
       </c>
       <c r="E47" t="n">
         <v>0</v>
       </c>
       <c r="F47" t="n">
-        <v>-2855268888.074034</v>
+        <v>-3425924546.32583</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -2199,7 +2199,7 @@
         </is>
       </c>
       <c r="H47" t="n">
-        <v>-2855268888.074034</v>
+        <v>-3425924546.32583</v>
       </c>
     </row>
     <row r="48">
@@ -2219,13 +2219,13 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>-1519913156.083462</v>
+        <v>-1785422281.217342</v>
       </c>
       <c r="E48" t="n">
-        <v>-89228971.64735198</v>
+        <v>-21440767.41358601</v>
       </c>
       <c r="F48" t="n">
-        <v>-1609142127.730814</v>
+        <v>-1806863048.630928</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -2233,7 +2233,7 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>-1609142127.730814</v>
+        <v>-1806863048.630928</v>
       </c>
     </row>
     <row r="49">
@@ -2253,13 +2253,13 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>-1502905845.684578</v>
+        <v>-1700162088.542067</v>
       </c>
       <c r="E49" t="n">
-        <v>-67395564.38218579</v>
+        <v>-68192336.54847036</v>
       </c>
       <c r="F49" t="n">
-        <v>-1570301410.066764</v>
+        <v>-1768354425.090537</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -2267,7 +2267,7 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>-1570301410.066764</v>
+        <v>-1768354425.090537</v>
       </c>
     </row>
     <row r="50">
@@ -2287,13 +2287,13 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>953915290.4645797</v>
+        <v>1034152271.827784</v>
       </c>
       <c r="E50" t="n">
-        <v>192642209.7906418</v>
+        <v>234613207.1805071</v>
       </c>
       <c r="F50" t="n">
-        <v>1146557500.255222</v>
+        <v>1268765479.008291</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -2301,7 +2301,7 @@
         </is>
       </c>
       <c r="H50" t="n">
-        <v>1146557500.255222</v>
+        <v>1268765479.008291</v>
       </c>
     </row>
     <row r="51">
@@ -2321,13 +2321,13 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>333904534.6795402</v>
+        <v>258183705.0118565</v>
       </c>
       <c r="E51" t="n">
-        <v>41073509.15706834</v>
+        <v>87750169.35835026</v>
       </c>
       <c r="F51" t="n">
-        <v>374978043.8366085</v>
+        <v>345933874.3702068</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -2335,7 +2335,7 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>374978043.8366085</v>
+        <v>345933874.3702068</v>
       </c>
     </row>
     <row r="52">
@@ -2358,10 +2358,10 @@
         <v>0</v>
       </c>
       <c r="E52" t="n">
-        <v>197454131.6721421</v>
+        <v>50838711.81797314</v>
       </c>
       <c r="F52" t="n">
-        <v>197454131.6721421</v>
+        <v>50838711.81797314</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -2369,7 +2369,7 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>197454131.6721421</v>
+        <v>50838711.81797314</v>
       </c>
     </row>
     <row r="53">
@@ -2392,10 +2392,10 @@
         <v>0</v>
       </c>
       <c r="E53" t="n">
-        <v>-203416267.7451056</v>
+        <v>-58878591.88523157</v>
       </c>
       <c r="F53" t="n">
-        <v>-203416267.7451056</v>
+        <v>-58878591.88523157</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -2403,7 +2403,7 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>-203416267.7451056</v>
+        <v>-58878591.88523157</v>
       </c>
     </row>
     <row r="54">
@@ -2423,13 +2423,13 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>1894798207.770339</v>
+        <v>1378172954.719548</v>
       </c>
       <c r="E54" t="n">
-        <v>576901289.4294164</v>
+        <v>393108003.7875938</v>
       </c>
       <c r="F54" t="n">
-        <v>2471699497.199755</v>
+        <v>1771280958.507141</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -2437,7 +2437,7 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>2471699497.199755</v>
+        <v>1771280958.507141</v>
       </c>
     </row>
     <row r="55">
@@ -2457,13 +2457,13 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>3370963813.785583</v>
+        <v>4393845235.142068</v>
       </c>
       <c r="E55" t="n">
-        <v>1128795126.66231</v>
+        <v>1434164354.392908</v>
       </c>
       <c r="F55" t="n">
-        <v>4499758940.447893</v>
+        <v>5828009589.534976</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -2471,7 +2471,7 @@
         </is>
       </c>
       <c r="H55" t="n">
-        <v>4499758940.447893</v>
+        <v>5828009589.534976</v>
       </c>
     </row>
     <row r="56">
@@ -2491,13 +2491,13 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>-2904978033.370792</v>
+        <v>-3478389930.401731</v>
       </c>
       <c r="E56" t="n">
         <v>0</v>
       </c>
       <c r="F56" t="n">
-        <v>-2904978033.370792</v>
+        <v>-3478389930.401731</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
@@ -2505,7 +2505,7 @@
         </is>
       </c>
       <c r="H56" t="n">
-        <v>-2904978033.370792</v>
+        <v>-3478389930.401731</v>
       </c>
     </row>
     <row r="57">
@@ -2525,13 +2525,13 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>-1520627674.7663</v>
+        <v>-1778660146.574771</v>
       </c>
       <c r="E57" t="n">
-        <v>-88985044.25020009</v>
+        <v>-21340537.19422145</v>
       </c>
       <c r="F57" t="n">
-        <v>-1609612719.0165</v>
+        <v>-1800000683.768992</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -2539,7 +2539,7 @@
         </is>
       </c>
       <c r="H57" t="n">
-        <v>-1609612719.0165</v>
+        <v>-1800000683.768992</v>
       </c>
     </row>
     <row r="58">
@@ -2559,13 +2559,13 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>-1511901728.280483</v>
+        <v>-1708782091.319164</v>
       </c>
       <c r="E58" t="n">
-        <v>-61887173.11008355</v>
+        <v>-62700575.33887476</v>
       </c>
       <c r="F58" t="n">
-        <v>-1573788901.390567</v>
+        <v>-1771482666.658039</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -2573,7 +2573,7 @@
         </is>
       </c>
       <c r="H58" t="n">
-        <v>-1573788901.390567</v>
+        <v>-1771482666.658039</v>
       </c>
     </row>
     <row r="59">
@@ -2593,13 +2593,13 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>974437567.7038515</v>
+        <v>1057149613.449686</v>
       </c>
       <c r="E59" t="n">
-        <v>194756216.1749827</v>
+        <v>237162249.3983841</v>
       </c>
       <c r="F59" t="n">
-        <v>1169193783.878834</v>
+        <v>1294311862.84807</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -2607,7 +2607,7 @@
         </is>
       </c>
       <c r="H59" t="n">
-        <v>1169193783.878834</v>
+        <v>1294311862.84807</v>
       </c>
     </row>
     <row r="60">
@@ -2627,13 +2627,13 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>336990611.6534101</v>
+        <v>271493772.2397426</v>
       </c>
       <c r="E60" t="n">
-        <v>36186933.31815184</v>
+        <v>72502667.67181981</v>
       </c>
       <c r="F60" t="n">
-        <v>373177544.971562</v>
+        <v>343996439.9115624</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -2641,7 +2641,7 @@
         </is>
       </c>
       <c r="H60" t="n">
-        <v>373177544.971562</v>
+        <v>343996439.9115624</v>
       </c>
     </row>
     <row r="61">
@@ -2664,10 +2664,10 @@
         <v>0</v>
       </c>
       <c r="E61" t="n">
-        <v>198151952.156349</v>
+        <v>51159562.05996025</v>
       </c>
       <c r="F61" t="n">
-        <v>198151952.156349</v>
+        <v>51159562.05996025</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -2675,7 +2675,7 @@
         </is>
       </c>
       <c r="H61" t="n">
-        <v>198151952.156349</v>
+        <v>51159562.05996025</v>
       </c>
     </row>
     <row r="62">
@@ -2698,10 +2698,10 @@
         <v>0</v>
       </c>
       <c r="E62" t="n">
-        <v>-178503779.9571419</v>
+        <v>-50327537.70444436</v>
       </c>
       <c r="F62" t="n">
-        <v>-178503779.9571419</v>
+        <v>-50327537.70444436</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -2709,7 +2709,7 @@
         </is>
       </c>
       <c r="H62" t="n">
-        <v>-178503779.9571419</v>
+        <v>-50327537.70444436</v>
       </c>
     </row>
     <row r="63">
@@ -2729,13 +2729,13 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>1932660886.371517</v>
+        <v>1404698533.360361</v>
       </c>
       <c r="E63" t="n">
-        <v>583805212.310558</v>
+        <v>397656888.5861675</v>
       </c>
       <c r="F63" t="n">
-        <v>2516466098.682075</v>
+        <v>1802355421.946528</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -2743,7 +2743,7 @@
         </is>
       </c>
       <c r="H63" t="n">
-        <v>2516466098.682075</v>
+        <v>1802355421.946528</v>
       </c>
     </row>
     <row r="64">
@@ -2763,13 +2763,13 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>3461142416.206189</v>
+        <v>4505195751.932012</v>
       </c>
       <c r="E64" t="n">
-        <v>1030611728.743424</v>
+        <v>1314111931.984749</v>
       </c>
       <c r="F64" t="n">
-        <v>4491754144.949613</v>
+        <v>5819307683.91676</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -2777,7 +2777,7 @@
         </is>
       </c>
       <c r="H64" t="n">
-        <v>4491754144.949613</v>
+        <v>5819307683.91676</v>
       </c>
     </row>
   </sheetData>
@@ -2848,13 +2848,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>465345192.4220803</v>
+        <v>-144251662.1232575</v>
       </c>
       <c r="C2" t="n">
-        <v>1824231668.883123</v>
+        <v>2233131347.127573</v>
       </c>
       <c r="D2" t="n">
-        <v>2289576861.305203</v>
+        <v>2088879685.004316</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -2862,16 +2862,16 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>-134741169.3209324</v>
+        <v>-85376944.77949929</v>
       </c>
       <c r="G2" t="n">
-        <v>-8.421323082558274</v>
+        <v>-7.114745398291608</v>
       </c>
       <c r="H2" t="n">
-        <v>-134741169.3209324</v>
+        <v>-85376944.77949929</v>
       </c>
       <c r="I2" t="n">
-        <v>-8.421323082558274</v>
+        <v>-7.114745398291608</v>
       </c>
     </row>
     <row r="3">
@@ -2881,13 +2881,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>916444004.9789721</v>
+        <v>475442510.2904696</v>
       </c>
       <c r="C3" t="n">
-        <v>1654490758.734831</v>
+        <v>1791770422.837109</v>
       </c>
       <c r="D3" t="n">
-        <v>2570934763.713802</v>
+        <v>2267212933.127579</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -2895,16 +2895,16 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>146616733.0876665</v>
+        <v>92956303.34376431</v>
       </c>
       <c r="G3" t="n">
-        <v>9.163545817979157</v>
+        <v>7.746358611980359</v>
       </c>
       <c r="H3" t="n">
-        <v>73308366.54383326</v>
+        <v>46478151.67188215</v>
       </c>
       <c r="I3" t="n">
-        <v>4.581772908989579</v>
+        <v>3.873179305990179</v>
       </c>
     </row>
     <row r="4">
@@ -2914,13 +2914,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>558382947.2380811</v>
+        <v>-8593058.749476984</v>
       </c>
       <c r="C4" t="n">
-        <v>1820161228.20051</v>
+        <v>2166960127.772038</v>
       </c>
       <c r="D4" t="n">
-        <v>2378544175.43859</v>
+        <v>2158367069.022562</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -2928,16 +2928,16 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>-45773855.18754578</v>
+        <v>-15889560.76125336</v>
       </c>
       <c r="G4" t="n">
-        <v>-2.860865949221611</v>
+        <v>-1.32413006343778</v>
       </c>
       <c r="H4" t="n">
-        <v>-45773855.18754578</v>
+        <v>-15889560.76125336</v>
       </c>
       <c r="I4" t="n">
-        <v>-2.860865949221611</v>
+        <v>-1.32413006343778</v>
       </c>
     </row>
     <row r="5">
@@ -2947,13 +2947,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>779194312.784005</v>
+        <v>280961236.1696404</v>
       </c>
       <c r="C5" t="n">
-        <v>1678902422.805181</v>
+        <v>1900974766.689718</v>
       </c>
       <c r="D5" t="n">
-        <v>2458096735.589186</v>
+        <v>2181936002.859358</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -2961,16 +2961,16 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>33778704.96305037</v>
+        <v>7679373.075543404</v>
       </c>
       <c r="G5" t="n">
-        <v>2.111169060190648</v>
+        <v>0.6399477562952836</v>
       </c>
       <c r="H5" t="n">
-        <v>16889352.48152518</v>
+        <v>3839686.537771702</v>
       </c>
       <c r="I5" t="n">
-        <v>1.055584530095324</v>
+        <v>0.3199738781476418</v>
       </c>
     </row>
     <row r="6">
@@ -2980,13 +2980,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>675019895.1158938</v>
+        <v>139139834.0518155</v>
       </c>
       <c r="C6" t="n">
-        <v>1722380600.271318</v>
+        <v>2005960283.043716</v>
       </c>
       <c r="D6" t="n">
-        <v>2397400495.387212</v>
+        <v>2145100117.095532</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -2994,16 +2994,16 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>-26917535.23892403</v>
+        <v>-29156512.68828297</v>
       </c>
       <c r="G6" t="n">
-        <v>-1.682345952432752</v>
+        <v>-2.429709390690247</v>
       </c>
       <c r="H6" t="n">
-        <v>-26917535.23892403</v>
+        <v>-29156512.68828297</v>
       </c>
       <c r="I6" t="n">
-        <v>-1.682345952432752</v>
+        <v>-2.429709390690247</v>
       </c>
     </row>
     <row r="7">
@@ -3013,13 +3013,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>675493956.8579671</v>
+        <v>152845250.6160171</v>
       </c>
       <c r="C7" t="n">
-        <v>1776825462.936935</v>
+        <v>2051962750.690044</v>
       </c>
       <c r="D7" t="n">
-        <v>2452319419.794902</v>
+        <v>2204808001.306062</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -3027,16 +3027,16 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>28001389.1687665</v>
+        <v>30551371.52224684</v>
       </c>
       <c r="G7" t="n">
-        <v>1.750086823047906</v>
+        <v>2.545947626853903</v>
       </c>
       <c r="H7" t="n">
-        <v>14000694.58438325</v>
+        <v>15275685.76112342</v>
       </c>
       <c r="I7" t="n">
-        <v>0.8750434115239532</v>
+        <v>1.272973813426952</v>
       </c>
     </row>
     <row r="8">
@@ -3046,13 +3046,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>767724045.517392</v>
+        <v>272705502.6861358</v>
       </c>
       <c r="C8" t="n">
-        <v>1714136045.38604</v>
+        <v>1938224649.46354</v>
       </c>
       <c r="D8" t="n">
-        <v>2481860090.903432</v>
+        <v>2210930152.149676</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -3060,16 +3060,16 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>57542060.27729654</v>
+        <v>36673522.36586094</v>
       </c>
       <c r="G8" t="n">
-        <v>3.596378767331034</v>
+        <v>3.056126863821745</v>
       </c>
       <c r="H8" t="n">
-        <v>28771030.13864827</v>
+        <v>18336761.18293047</v>
       </c>
       <c r="I8" t="n">
-        <v>1.798189383665517</v>
+        <v>1.528063431910873</v>
       </c>
     </row>
   </sheetData>

</xml_diff>